<commit_message>
add SMTP email reminder for unpaid invoices
</commit_message>
<xml_diff>
--- a/Data/Input/Invoice_Data.xlsx
+++ b/Data/Input/Invoice_Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Git-dbot24\UiPath-InvoiceReminderAutomation\Data\Input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C812542-B940-4B18-BE70-27C35FEF7768}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36B25BAF-5E0C-406A-973B-60A3A45D850C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,12 +16,12 @@
     <sheet name="Invoices" sheetId="1" r:id="rId1"/>
     <sheet name="Instructions" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="231">
   <si>
     <t>InvoiceID</t>
   </si>
@@ -705,6 +705,15 @@
   </si>
   <si>
     <t>Today's date for calculation reference: 2026-08-30</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>Medium</t>
   </si>
 </sst>
 </file>
@@ -1200,8 +1209,12 @@
       <c r="G2" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="8"/>
-      <c r="I2" s="2"/>
+      <c r="H2" s="8">
+        <v>42</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>228</v>
+      </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
@@ -1225,8 +1238,12 @@
       <c r="G3" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H3" s="8"/>
-      <c r="I3" s="2"/>
+      <c r="H3" s="8">
+        <v>81</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>228</v>
+      </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
@@ -1250,8 +1267,12 @@
       <c r="G4" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H4" s="8"/>
-      <c r="I4" s="2"/>
+      <c r="H4" s="8">
+        <v>27</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>228</v>
+      </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -1275,8 +1296,12 @@
       <c r="G5" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="8"/>
-      <c r="I5" s="2"/>
+      <c r="H5" s="8">
+        <v>70</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>228</v>
+      </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
@@ -1300,8 +1325,12 @@
       <c r="G6" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H6" s="8"/>
-      <c r="I6" s="2"/>
+      <c r="H6" s="8">
+        <v>58</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>228</v>
+      </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
@@ -1325,8 +1354,12 @@
       <c r="G7" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H7" s="8"/>
-      <c r="I7" s="2"/>
+      <c r="H7" s="8">
+        <v>59</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>228</v>
+      </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
@@ -1350,8 +1383,12 @@
       <c r="G8" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H8" s="8"/>
-      <c r="I8" s="2"/>
+      <c r="H8" s="8">
+        <v>69</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>228</v>
+      </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
@@ -1375,8 +1412,12 @@
       <c r="G9" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H9" s="8"/>
-      <c r="I9" s="2"/>
+      <c r="H9" s="8">
+        <v>54</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>228</v>
+      </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
@@ -1400,8 +1441,12 @@
       <c r="G10" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H10" s="8"/>
-      <c r="I10" s="2"/>
+      <c r="H10" s="8">
+        <v>17</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>228</v>
+      </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
@@ -1425,8 +1470,12 @@
       <c r="G11" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H11" s="8"/>
-      <c r="I11" s="2"/>
+      <c r="H11" s="8">
+        <v>55</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>228</v>
+      </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
@@ -1450,7 +1499,9 @@
       <c r="G12" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="H12" s="9"/>
+      <c r="H12" s="9">
+        <v>0</v>
+      </c>
       <c r="I12" s="2"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
@@ -1475,8 +1526,12 @@
       <c r="G13" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H13" s="8"/>
-      <c r="I13" s="2"/>
+      <c r="H13" s="8">
+        <v>41</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>228</v>
+      </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
@@ -1500,8 +1555,12 @@
       <c r="G14" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H14" s="8"/>
-      <c r="I14" s="2"/>
+      <c r="H14" s="8">
+        <v>42</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>228</v>
+      </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
@@ -1525,7 +1584,9 @@
       <c r="G15" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="H15" s="9"/>
+      <c r="H15" s="9">
+        <v>0</v>
+      </c>
       <c r="I15" s="2"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
@@ -1550,8 +1611,12 @@
       <c r="G16" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H16" s="8"/>
-      <c r="I16" s="2"/>
+      <c r="H16" s="8">
+        <v>37</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>228</v>
+      </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
@@ -1575,8 +1640,12 @@
       <c r="G17" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H17" s="8"/>
-      <c r="I17" s="2"/>
+      <c r="H17" s="8">
+        <v>15</v>
+      </c>
+      <c r="I17" s="2" t="s">
+        <v>228</v>
+      </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
@@ -1600,8 +1669,12 @@
       <c r="G18" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H18" s="8"/>
-      <c r="I18" s="2"/>
+      <c r="H18" s="8">
+        <v>21</v>
+      </c>
+      <c r="I18" s="2" t="s">
+        <v>228</v>
+      </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
@@ -1625,8 +1698,12 @@
       <c r="G19" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H19" s="8"/>
-      <c r="I19" s="2"/>
+      <c r="H19" s="8">
+        <v>73</v>
+      </c>
+      <c r="I19" s="2" t="s">
+        <v>228</v>
+      </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
@@ -1650,8 +1727,12 @@
       <c r="G20" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H20" s="8"/>
-      <c r="I20" s="2"/>
+      <c r="H20" s="8">
+        <v>38</v>
+      </c>
+      <c r="I20" s="2" t="s">
+        <v>228</v>
+      </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
@@ -1675,8 +1756,12 @@
       <c r="G21" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H21" s="8"/>
-      <c r="I21" s="2"/>
+      <c r="H21" s="8">
+        <v>31</v>
+      </c>
+      <c r="I21" s="2" t="s">
+        <v>228</v>
+      </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
@@ -1700,8 +1785,12 @@
       <c r="G22" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H22" s="8"/>
-      <c r="I22" s="2"/>
+      <c r="H22" s="8">
+        <v>72</v>
+      </c>
+      <c r="I22" s="2" t="s">
+        <v>228</v>
+      </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
@@ -1725,8 +1814,12 @@
       <c r="G23" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H23" s="8"/>
-      <c r="I23" s="2"/>
+      <c r="H23" s="8">
+        <v>4</v>
+      </c>
+      <c r="I23" s="2" t="s">
+        <v>229</v>
+      </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
@@ -1750,8 +1843,12 @@
       <c r="G24" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H24" s="8"/>
-      <c r="I24" s="2"/>
+      <c r="H24" s="8">
+        <v>14</v>
+      </c>
+      <c r="I24" s="2" t="s">
+        <v>230</v>
+      </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
@@ -1775,7 +1872,9 @@
       <c r="G25" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="H25" s="9"/>
+      <c r="H25" s="9">
+        <v>0</v>
+      </c>
       <c r="I25" s="2"/>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.3">
@@ -1800,8 +1899,12 @@
       <c r="G26" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H26" s="8"/>
-      <c r="I26" s="2"/>
+      <c r="H26" s="8">
+        <v>68</v>
+      </c>
+      <c r="I26" s="2" t="s">
+        <v>228</v>
+      </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
@@ -1825,8 +1928,12 @@
       <c r="G27" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H27" s="8"/>
-      <c r="I27" s="2"/>
+      <c r="H27" s="8">
+        <v>54</v>
+      </c>
+      <c r="I27" s="2" t="s">
+        <v>228</v>
+      </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
@@ -1850,7 +1957,9 @@
       <c r="G28" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="H28" s="9"/>
+      <c r="H28" s="9">
+        <v>0</v>
+      </c>
       <c r="I28" s="2"/>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.3">
@@ -1875,7 +1984,9 @@
       <c r="G29" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="H29" s="9"/>
+      <c r="H29" s="9">
+        <v>0</v>
+      </c>
       <c r="I29" s="2"/>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.3">
@@ -1900,8 +2011,12 @@
       <c r="G30" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H30" s="8"/>
-      <c r="I30" s="2"/>
+      <c r="H30" s="8">
+        <v>54</v>
+      </c>
+      <c r="I30" s="2" t="s">
+        <v>228</v>
+      </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
@@ -1925,8 +2040,12 @@
       <c r="G31" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H31" s="8"/>
-      <c r="I31" s="2"/>
+      <c r="H31" s="8">
+        <v>15</v>
+      </c>
+      <c r="I31" s="2" t="s">
+        <v>228</v>
+      </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
@@ -1950,8 +2069,12 @@
       <c r="G32" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H32" s="8"/>
-      <c r="I32" s="2"/>
+      <c r="H32" s="8">
+        <v>58</v>
+      </c>
+      <c r="I32" s="2" t="s">
+        <v>228</v>
+      </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
@@ -1975,7 +2098,9 @@
       <c r="G33" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="H33" s="9"/>
+      <c r="H33" s="9">
+        <v>0</v>
+      </c>
       <c r="I33" s="2"/>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.3">
@@ -2000,8 +2125,12 @@
       <c r="G34" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H34" s="8"/>
-      <c r="I34" s="2"/>
+      <c r="H34" s="8">
+        <v>24</v>
+      </c>
+      <c r="I34" s="2" t="s">
+        <v>228</v>
+      </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
@@ -2025,8 +2154,12 @@
       <c r="G35" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H35" s="8"/>
-      <c r="I35" s="2"/>
+      <c r="H35" s="8">
+        <v>9</v>
+      </c>
+      <c r="I35" s="2" t="s">
+        <v>230</v>
+      </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
@@ -2050,8 +2183,12 @@
       <c r="G36" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H36" s="8"/>
-      <c r="I36" s="2"/>
+      <c r="H36" s="8">
+        <v>13</v>
+      </c>
+      <c r="I36" s="2" t="s">
+        <v>230</v>
+      </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
@@ -2075,8 +2212,12 @@
       <c r="G37" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H37" s="8"/>
-      <c r="I37" s="2"/>
+      <c r="H37" s="8">
+        <v>29</v>
+      </c>
+      <c r="I37" s="2" t="s">
+        <v>228</v>
+      </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
@@ -2100,7 +2241,9 @@
       <c r="G38" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="H38" s="9"/>
+      <c r="H38" s="9">
+        <v>0</v>
+      </c>
       <c r="I38" s="2"/>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.3">
@@ -2125,8 +2268,12 @@
       <c r="G39" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H39" s="8"/>
-      <c r="I39" s="2"/>
+      <c r="H39" s="8">
+        <v>72</v>
+      </c>
+      <c r="I39" s="2" t="s">
+        <v>228</v>
+      </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
@@ -2150,8 +2297,12 @@
       <c r="G40" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H40" s="8"/>
-      <c r="I40" s="2"/>
+      <c r="H40" s="8">
+        <v>82</v>
+      </c>
+      <c r="I40" s="2" t="s">
+        <v>228</v>
+      </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
@@ -2175,8 +2326,12 @@
       <c r="G41" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H41" s="8"/>
-      <c r="I41" s="2"/>
+      <c r="H41" s="8">
+        <v>62</v>
+      </c>
+      <c r="I41" s="2" t="s">
+        <v>228</v>
+      </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
@@ -2200,8 +2355,12 @@
       <c r="G42" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H42" s="8"/>
-      <c r="I42" s="2"/>
+      <c r="H42" s="8">
+        <v>15</v>
+      </c>
+      <c r="I42" s="2" t="s">
+        <v>228</v>
+      </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
@@ -2225,7 +2384,9 @@
       <c r="G43" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="H43" s="9"/>
+      <c r="H43" s="9">
+        <v>0</v>
+      </c>
       <c r="I43" s="2"/>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.3">
@@ -2250,8 +2411,12 @@
       <c r="G44" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H44" s="8"/>
-      <c r="I44" s="2"/>
+      <c r="H44" s="8">
+        <v>30</v>
+      </c>
+      <c r="I44" s="2" t="s">
+        <v>228</v>
+      </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
@@ -2275,7 +2440,9 @@
       <c r="G45" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="H45" s="9"/>
+      <c r="H45" s="9">
+        <v>0</v>
+      </c>
       <c r="I45" s="2"/>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.3">
@@ -2300,8 +2467,12 @@
       <c r="G46" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H46" s="8"/>
-      <c r="I46" s="2"/>
+      <c r="H46" s="8">
+        <v>24</v>
+      </c>
+      <c r="I46" s="2" t="s">
+        <v>228</v>
+      </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
@@ -2325,8 +2496,12 @@
       <c r="G47" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H47" s="8"/>
-      <c r="I47" s="2"/>
+      <c r="H47" s="8">
+        <v>15</v>
+      </c>
+      <c r="I47" s="2" t="s">
+        <v>228</v>
+      </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
@@ -2350,7 +2525,9 @@
       <c r="G48" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="H48" s="9"/>
+      <c r="H48" s="9">
+        <v>0</v>
+      </c>
       <c r="I48" s="2"/>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.3">
@@ -2375,8 +2552,12 @@
       <c r="G49" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H49" s="8"/>
-      <c r="I49" s="2"/>
+      <c r="H49" s="8">
+        <v>23</v>
+      </c>
+      <c r="I49" s="2" t="s">
+        <v>228</v>
+      </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
@@ -2400,8 +2581,12 @@
       <c r="G50" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H50" s="8"/>
-      <c r="I50" s="2"/>
+      <c r="H50" s="8">
+        <v>44</v>
+      </c>
+      <c r="I50" s="2" t="s">
+        <v>228</v>
+      </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
@@ -2425,7 +2610,9 @@
       <c r="G51" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="H51" s="9"/>
+      <c r="H51" s="9">
+        <v>0</v>
+      </c>
       <c r="I51" s="2"/>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.3">

</xml_diff>